<commit_message>
Add sample adequacy and pilot clarity patch
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/real_student_online_5case_coach_review_form_cn_v2.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/real_student_online_5case_coach_review_form_cn_v2.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50-case字段对照" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'教练复核表'!$A$1:$AM$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'教练复核表'!$A$1:$AV$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -244,47 +244,77 @@
     <author>Codex</author>
   </authors>
   <commentList>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>不要填写真实学生身份。可填写题目名、匿名题号或内部脱敏题目标识。</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>人工改写的任务摘要，不粘贴完整题面。用于判断 context sufficiency 和 rubric transfer。</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>只保留足以判断当前 missing bridge 的约束、输入输出或目标摘要。</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>概括学生已经知道什么、当前卡在哪里。不要粘贴完整私有对话。</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>判断当前摘要是否足够教练评分；不足时应降低复核信心或要求查看完整题面。</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>固定说明：这是线上已经展示给学生的 observed current-system response，不是 7 个 offline conditions 中的实验条件。</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: coach_bridge_identification_score。2=准确抓住；1=部分抓住；0=没抓住。</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: coach_groundedness_score。看回复是否基于题目、学生话语和近期对话。</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: coach_scaffold_appropriateness_score。太弱、太强、直接给答案都扣分。</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: coach_bridge_leakage_control_score。0=严重泄露，1=边界/轻微，2=控制良好。</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="AE1" authorId="0" shapeId="0">
       <text>
-        <t>对齐 50-case: coach_leakage_label。判断当前 AIChat 是否提前补完 critical bridge。</t>
+        <t>对齐 50-case: coach_leakage_label。判断 observed current AIChat response 是否提前补完 critical bridge；它是观察项，非实验条件。</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="AF1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: coach_overall_quality_score。1=不可用，5=很适合给学生。</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: coach_would_show_to_student。</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <t>对齐 50-case: student_response_burden。低=短回复即可，高=完整推导/表格/代码。</t>
       </text>
     </comment>
-    <comment ref="AL1" authorId="0" shapeId="0">
+    <comment ref="AU1" authorId="0" shapeId="0">
       <text>
         <t>未完成前保持“待完成”。不是“可报告”时，不能写成公开 deep-pilot evidence。</t>
       </text>
@@ -582,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -616,58 +646,82 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>评分区</t>
+          <t>题目上下文字段</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>7 个 0/1/2 小分、泄露标签、总体质量、是否愿意给学生看、学生回答负担等，均对齐 50-case 人审口径。</t>
+          <t>题目任务摘要、关键约束/输入输出摘要、当前学生状态摘要用于判断 context sufficiency 和 rubric transfer；不要粘贴完整题面。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Pilot validity 区</t>
+          <t>当前AIChat回复字段</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>缺失桥家族、当前缺失桥实例、禁止内容、可提示边界、期望学生下一步，用于检查 taxonomy/rubric 是否能迁移到真实学生对话。</t>
+          <t>“当前AIChat回复（已脱敏）”是线上已展示回复，观察项，非实验条件；不要把它写成 baseline、condition 或 control。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>隐私边界</t>
+          <t>评分区</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>不要把完整学生原文、完整代码、完整 AI 回复复制到公开材料。私有工作簿只保存在 .local_private。</t>
+          <t>7 个 0/1/2 小分、泄露标签、总体质量、是否愿意给学生看、学生回答负担等，均对齐 50-case 人审口径。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>知情/报告门</t>
+          <t>Pilot validity 区</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>保持“待完成”时，不能把该 case 写成公开 deep-pilot evidence。</t>
+          <t>缺失桥家族、当前缺失桥实例、禁止内容、可提示边界、期望学生下一步，用于检查 taxonomy/rubric 是否能迁移到真实学生对话。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>隐私边界</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>不要把完整学生原文、完整代码、完整 AI 回复复制到公开材料。私有工作簿只保存在 .local_private。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>知情/报告门</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>保持“待完成”时，不能把该 case 写成公开 deep-pilot evidence。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>颜色提示</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>绿色通常表示较安全/较好，黄色表示边界/待完成，红色表示高风险/低分，灰色表示不可报告或不适用。</t>
         </is>
@@ -684,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM6"/>
+  <dimension ref="A1:AV6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -692,40 +746,49 @@
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="36" customWidth="1" min="29" max="29"/>
-    <col width="36" customWidth="1" min="30" max="30"/>
-    <col width="36" customWidth="1" min="31" max="31"/>
-    <col width="34" customWidth="1" min="32" max="32"/>
-    <col width="18" customWidth="1" min="33" max="33"/>
-    <col width="20" customWidth="1" min="34" max="34"/>
-    <col width="16" customWidth="1" min="35" max="35"/>
-    <col width="16" customWidth="1" min="36" max="36"/>
-    <col width="14" customWidth="1" min="37" max="37"/>
-    <col width="14" customWidth="1" min="38" max="38"/>
-    <col width="40" customWidth="1" min="39" max="39"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
+    <col width="48" customWidth="1" min="16" max="16"/>
+    <col width="44" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="48" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="14" customWidth="1" min="36" max="36"/>
+    <col width="22" customWidth="1" min="37" max="37"/>
+    <col width="36" customWidth="1" min="38" max="38"/>
+    <col width="36" customWidth="1" min="39" max="39"/>
+    <col width="36" customWidth="1" min="40" max="40"/>
+    <col width="34" customWidth="1" min="41" max="41"/>
+    <col width="18" customWidth="1" min="42" max="42"/>
+    <col width="20" customWidth="1" min="43" max="43"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
+    <col width="16" customWidth="1" min="45" max="45"/>
+    <col width="14" customWidth="1" min="46" max="46"/>
+    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="40" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -756,170 +819,215 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
+          <t>题目名称/匿名题号</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>题目任务摘要</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>关键约束/输入输出摘要</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>当前学生状态摘要</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>是否有完整题目上下文</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>题目摘要是否足够评分</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>是否需要查看完整题面才能评分</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>题目摘要来源</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
           <t>题目/场景摘要</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>学生问题（已脱敏）</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>近期对话（已脱敏，可空）</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>学生代码片段（已脱敏，可空）</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>当前AIChat回复字段说明</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>当前AIChat回复（已脱敏）</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>复核状态</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>隐私复核状态</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>上下文是否足够</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>识别当前缺失桥是否准确（0/1/2）</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="X1" s="7" t="inlineStr">
         <is>
           <t>回复是否基于当前材料（0/1/2）</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="Y1" s="7" t="inlineStr">
         <is>
           <t>脚手架是否合适（0/1/2）</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="Z1" s="7" t="inlineStr">
         <is>
           <t>是否控制关键桥泄露（0/1/2）</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>下一步是否清楚（0/1/2）</t>
         </is>
       </c>
-      <c r="S1" s="7" t="inlineStr">
+      <c r="AB1" s="7" t="inlineStr">
         <is>
           <t>是否单焦点连贯（0/1/2）</t>
         </is>
       </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="AC1" s="7" t="inlineStr">
         <is>
           <t>微例是否围绕桥梁（0/1/2/不适用）</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="AD1" s="7" t="inlineStr">
         <is>
           <t>微例适用性</t>
         </is>
       </c>
-      <c r="V1" s="7" t="inlineStr">
+      <c r="AE1" s="7" t="inlineStr">
         <is>
           <t>泄露标签</t>
         </is>
       </c>
-      <c r="W1" s="7" t="inlineStr">
+      <c r="AF1" s="7" t="inlineStr">
         <is>
           <t>总体质量（1-5）</t>
         </is>
       </c>
-      <c r="X1" s="7" t="inlineStr">
+      <c r="AG1" s="7" t="inlineStr">
         <is>
           <t>是否愿意给学生看</t>
         </is>
       </c>
-      <c r="Y1" s="7" t="inlineStr">
+      <c r="AH1" s="7" t="inlineStr">
         <is>
           <t>学生回答负担</t>
         </is>
       </c>
-      <c r="Z1" s="7" t="inlineStr">
+      <c r="AI1" s="7" t="inlineStr">
         <is>
           <t>复核信心</t>
         </is>
       </c>
-      <c r="AA1" s="7" t="inlineStr">
+      <c r="AJ1" s="7" t="inlineStr">
         <is>
           <t>是否需要讨论</t>
         </is>
       </c>
-      <c r="AB1" s="8" t="inlineStr">
+      <c r="AK1" s="8" t="inlineStr">
         <is>
           <t>缺失桥家族（中文）</t>
         </is>
       </c>
-      <c r="AC1" s="8" t="inlineStr">
+      <c r="AL1" s="8" t="inlineStr">
         <is>
           <t>当前缺失桥实例（中文简述）</t>
         </is>
       </c>
-      <c r="AD1" s="8" t="inlineStr">
+      <c r="AM1" s="8" t="inlineStr">
         <is>
           <t>禁止直接说出的内容（中文）</t>
         </is>
       </c>
-      <c r="AE1" s="8" t="inlineStr">
+      <c r="AN1" s="8" t="inlineStr">
         <is>
           <t>可以提示到什么程度（中文）</t>
         </is>
       </c>
-      <c r="AF1" s="8" t="inlineStr">
+      <c r="AO1" s="8" t="inlineStr">
         <is>
           <t>期望学生下一步（中文）</t>
         </is>
       </c>
-      <c r="AG1" s="8" t="inlineStr">
+      <c r="AP1" s="8" t="inlineStr">
         <is>
           <t>是否匹配现有taxonomy</t>
         </is>
       </c>
-      <c r="AH1" s="8" t="inlineStr">
+      <c r="AQ1" s="8" t="inlineStr">
         <is>
           <t>新桥候选（如无填“无”）</t>
         </is>
       </c>
-      <c r="AI1" s="8" t="inlineStr">
+      <c r="AR1" s="8" t="inlineStr">
         <is>
           <t>观察到的下一轮进展</t>
         </is>
       </c>
-      <c r="AJ1" s="8" t="inlineStr">
+      <c r="AS1" s="8" t="inlineStr">
         <is>
           <t>是否同意AI预标注</t>
         </is>
       </c>
-      <c r="AK1" s="8" t="inlineStr">
+      <c r="AT1" s="8" t="inlineStr">
         <is>
           <t>是否需要裁决</t>
         </is>
       </c>
-      <c r="AL1" s="6" t="inlineStr">
+      <c r="AU1" s="6" t="inlineStr">
         <is>
           <t>知情/报告门</t>
         </is>
       </c>
-      <c r="AM1" s="9" t="inlineStr">
+      <c r="AV1" s="9" t="inlineStr">
         <is>
           <t>教练备注（中文）</t>
         </is>
@@ -958,43 +1066,79 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
+          <t>见本地私有表；公开模板不含完整题面</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；仅保留足以判断当前卡点的改写摘要</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；由教练用中文概括</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>线上AIChat元数据</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>线上已展示回复，观察项，非实验条件</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr"/>
-      <c r="Q2" s="4" t="inlineStr"/>
-      <c r="R2" s="4" t="inlineStr"/>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
       <c r="V2" s="4" t="inlineStr"/>
       <c r="W2" s="4" t="inlineStr"/>
       <c r="X2" s="4" t="inlineStr"/>
@@ -1011,12 +1155,21 @@
       <c r="AI2" s="4" t="inlineStr"/>
       <c r="AJ2" s="4" t="inlineStr"/>
       <c r="AK2" s="4" t="inlineStr"/>
-      <c r="AL2" s="4" t="inlineStr">
+      <c r="AL2" s="4" t="inlineStr"/>
+      <c r="AM2" s="4" t="inlineStr"/>
+      <c r="AN2" s="4" t="inlineStr"/>
+      <c r="AO2" s="4" t="inlineStr"/>
+      <c r="AP2" s="4" t="inlineStr"/>
+      <c r="AQ2" s="4" t="inlineStr"/>
+      <c r="AR2" s="4" t="inlineStr"/>
+      <c r="AS2" s="4" t="inlineStr"/>
+      <c r="AT2" s="4" t="inlineStr"/>
+      <c r="AU2" s="4" t="inlineStr">
         <is>
           <t>待完成</t>
         </is>
       </c>
-      <c r="AM2" s="4" t="inlineStr"/>
+      <c r="AV2" s="4" t="inlineStr"/>
     </row>
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -1051,43 +1204,79 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
+          <t>见本地私有表；公开模板不含完整题面</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；仅保留足以判断当前卡点的改写摘要</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；由教练用中文概括</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>线上AIChat元数据</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>线上已展示回复，观察项，非实验条件</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="U3" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
-      <c r="Q3" s="4" t="inlineStr"/>
-      <c r="R3" s="4" t="inlineStr"/>
-      <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
       <c r="V3" s="4" t="inlineStr"/>
       <c r="W3" s="4" t="inlineStr"/>
       <c r="X3" s="4" t="inlineStr"/>
@@ -1104,12 +1293,21 @@
       <c r="AI3" s="4" t="inlineStr"/>
       <c r="AJ3" s="4" t="inlineStr"/>
       <c r="AK3" s="4" t="inlineStr"/>
-      <c r="AL3" s="4" t="inlineStr">
+      <c r="AL3" s="4" t="inlineStr"/>
+      <c r="AM3" s="4" t="inlineStr"/>
+      <c r="AN3" s="4" t="inlineStr"/>
+      <c r="AO3" s="4" t="inlineStr"/>
+      <c r="AP3" s="4" t="inlineStr"/>
+      <c r="AQ3" s="4" t="inlineStr"/>
+      <c r="AR3" s="4" t="inlineStr"/>
+      <c r="AS3" s="4" t="inlineStr"/>
+      <c r="AT3" s="4" t="inlineStr"/>
+      <c r="AU3" s="4" t="inlineStr">
         <is>
           <t>待完成</t>
         </is>
       </c>
-      <c r="AM3" s="4" t="inlineStr"/>
+      <c r="AV3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -1144,43 +1342,79 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>见本地私有表；公开模板不含完整题面</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；仅保留足以判断当前卡点的改写摘要</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；由教练用中文概括</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>线上AIChat元数据</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>线上已展示回复，观察项，非实验条件</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr"/>
-      <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr"/>
-      <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr"/>
       <c r="V4" s="4" t="inlineStr"/>
       <c r="W4" s="4" t="inlineStr"/>
       <c r="X4" s="4" t="inlineStr"/>
@@ -1197,12 +1431,21 @@
       <c r="AI4" s="4" t="inlineStr"/>
       <c r="AJ4" s="4" t="inlineStr"/>
       <c r="AK4" s="4" t="inlineStr"/>
-      <c r="AL4" s="4" t="inlineStr">
+      <c r="AL4" s="4" t="inlineStr"/>
+      <c r="AM4" s="4" t="inlineStr"/>
+      <c r="AN4" s="4" t="inlineStr"/>
+      <c r="AO4" s="4" t="inlineStr"/>
+      <c r="AP4" s="4" t="inlineStr"/>
+      <c r="AQ4" s="4" t="inlineStr"/>
+      <c r="AR4" s="4" t="inlineStr"/>
+      <c r="AS4" s="4" t="inlineStr"/>
+      <c r="AT4" s="4" t="inlineStr"/>
+      <c r="AU4" s="4" t="inlineStr">
         <is>
           <t>待完成</t>
         </is>
       </c>
-      <c r="AM4" s="4" t="inlineStr"/>
+      <c r="AV4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1237,43 +1480,79 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>见本地私有表；公开模板不含完整题面</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；仅保留足以判断当前卡点的改写摘要</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；由教练用中文概括</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>线上AIChat元数据</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>线上已展示回复，观察项，非实验条件</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
-      <c r="Q5" s="4" t="inlineStr"/>
-      <c r="R5" s="4" t="inlineStr"/>
-      <c r="S5" s="4" t="inlineStr"/>
-      <c r="T5" s="4" t="inlineStr"/>
-      <c r="U5" s="4" t="inlineStr"/>
       <c r="V5" s="4" t="inlineStr"/>
       <c r="W5" s="4" t="inlineStr"/>
       <c r="X5" s="4" t="inlineStr"/>
@@ -1290,12 +1569,21 @@
       <c r="AI5" s="4" t="inlineStr"/>
       <c r="AJ5" s="4" t="inlineStr"/>
       <c r="AK5" s="4" t="inlineStr"/>
-      <c r="AL5" s="4" t="inlineStr">
+      <c r="AL5" s="4" t="inlineStr"/>
+      <c r="AM5" s="4" t="inlineStr"/>
+      <c r="AN5" s="4" t="inlineStr"/>
+      <c r="AO5" s="4" t="inlineStr"/>
+      <c r="AP5" s="4" t="inlineStr"/>
+      <c r="AQ5" s="4" t="inlineStr"/>
+      <c r="AR5" s="4" t="inlineStr"/>
+      <c r="AS5" s="4" t="inlineStr"/>
+      <c r="AT5" s="4" t="inlineStr"/>
+      <c r="AU5" s="4" t="inlineStr">
         <is>
           <t>待完成</t>
         </is>
       </c>
-      <c r="AM5" s="4" t="inlineStr"/>
+      <c r="AV5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -1330,43 +1618,79 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
+          <t>见本地私有表；公开模板不含完整题面</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；仅保留足以判断当前卡点的改写摘要</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表；由教练用中文概括</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>线上AIChat元数据</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>见本地私有表</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>线上已展示回复，观察项，非实验条件</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>见本地私有表</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
-      <c r="Q6" s="4" t="inlineStr"/>
-      <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="4" t="inlineStr"/>
-      <c r="T6" s="4" t="inlineStr"/>
-      <c r="U6" s="4" t="inlineStr"/>
       <c r="V6" s="4" t="inlineStr"/>
       <c r="W6" s="4" t="inlineStr"/>
       <c r="X6" s="4" t="inlineStr"/>
@@ -1383,16 +1707,25 @@
       <c r="AI6" s="4" t="inlineStr"/>
       <c r="AJ6" s="4" t="inlineStr"/>
       <c r="AK6" s="4" t="inlineStr"/>
-      <c r="AL6" s="4" t="inlineStr">
+      <c r="AL6" s="4" t="inlineStr"/>
+      <c r="AM6" s="4" t="inlineStr"/>
+      <c r="AN6" s="4" t="inlineStr"/>
+      <c r="AO6" s="4" t="inlineStr"/>
+      <c r="AP6" s="4" t="inlineStr"/>
+      <c r="AQ6" s="4" t="inlineStr"/>
+      <c r="AR6" s="4" t="inlineStr"/>
+      <c r="AS6" s="4" t="inlineStr"/>
+      <c r="AT6" s="4" t="inlineStr"/>
+      <c r="AU6" s="4" t="inlineStr">
         <is>
           <t>待完成</t>
         </is>
       </c>
-      <c r="AM6" s="4" t="inlineStr"/>
+      <c r="AV6" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM6"/>
-  <conditionalFormatting sqref="N2:N6">
+  <autoFilter ref="A1:AV6"/>
+  <conditionalFormatting sqref="W2:W6">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1403,7 +1736,7 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O6">
+  <conditionalFormatting sqref="X2:X6">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1414,7 +1747,7 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P6">
+  <conditionalFormatting sqref="Y2:Y6">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1425,7 +1758,7 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q6">
+  <conditionalFormatting sqref="Z2:Z6">
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1436,7 +1769,7 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R6">
+  <conditionalFormatting sqref="AA2:AA6">
     <cfRule type="cellIs" priority="13" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1447,7 +1780,7 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S6">
+  <conditionalFormatting sqref="AB2:AB6">
     <cfRule type="cellIs" priority="16" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1458,7 +1791,7 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T6">
+  <conditionalFormatting sqref="AC2:AC6">
     <cfRule type="cellIs" priority="19" operator="equal" dxfId="0">
       <formula>"2"</formula>
     </cfRule>
@@ -1469,118 +1802,129 @@
       <formula>"0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V6">
+  <conditionalFormatting sqref="AE2:AE6">
     <cfRule type="expression" priority="22" dxfId="0">
-      <formula>=$V2="无泄露"</formula>
+      <formula>=$AE2="无泄露"</formula>
     </cfRule>
     <cfRule type="expression" priority="23" dxfId="1">
-      <formula>=$V2="轻微关键桥泄露"</formula>
+      <formula>=$AE2="轻微关键桥泄露"</formula>
     </cfRule>
     <cfRule type="expression" priority="24" dxfId="2">
-      <formula>=OR($V2="重大关键桥泄露",$V2="答案或代码泄露")</formula>
+      <formula>=OR($AE2="重大关键桥泄露",$AE2="答案或代码泄露")</formula>
     </cfRule>
     <cfRule type="expression" priority="25" dxfId="3">
-      <formula>=$V2="上下文不足未判断"</formula>
+      <formula>=$AE2="上下文不足未判断"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:X6">
+  <conditionalFormatting sqref="AG2:AG6">
     <cfRule type="expression" priority="26" dxfId="0">
-      <formula>=$X2="是"</formula>
+      <formula>=$AG2="是"</formula>
     </cfRule>
     <cfRule type="expression" priority="27" dxfId="1">
-      <formula>=$X2="边界"</formula>
+      <formula>=$AG2="边界"</formula>
     </cfRule>
     <cfRule type="expression" priority="28" dxfId="2">
-      <formula>=$X2="否"</formula>
+      <formula>=$AG2="否"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y2:Y6">
+  <conditionalFormatting sqref="AH2:AH6">
     <cfRule type="expression" priority="29" dxfId="0">
-      <formula>=$Y2="低"</formula>
+      <formula>=$AH2="低"</formula>
     </cfRule>
     <cfRule type="expression" priority="30" dxfId="1">
-      <formula>=$Y2="中"</formula>
+      <formula>=$AH2="中"</formula>
     </cfRule>
     <cfRule type="expression" priority="31" dxfId="2">
-      <formula>=$Y2="高"</formula>
+      <formula>=$AH2="高"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL2:AL6">
+  <conditionalFormatting sqref="AU2:AU6">
     <cfRule type="expression" priority="32" dxfId="0">
-      <formula>=$AL2="可报告"</formula>
+      <formula>=$AU2="可报告"</formula>
     </cfRule>
     <cfRule type="expression" priority="33" dxfId="1">
-      <formula>=$AL2="待完成"</formula>
+      <formula>=$AU2="待完成"</formula>
     </cfRule>
     <cfRule type="expression" priority="34" dxfId="3">
-      <formula>=OR($AL2="不可报告",$AL2="已退出")</formula>
+      <formula>=OR($AU2="不可报告",$AU2="已退出")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W6">
-    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="0">
+  <conditionalFormatting sqref="K2:K6">
+    <cfRule type="expression" priority="35" dxfId="0">
+      <formula>=$K2="足够"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="36" dxfId="1">
+      <formula>=$K2="部分足够"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="37" dxfId="2">
+      <formula>=OR($K2="不足",$K2="不确定")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF2:AF6">
+    <cfRule type="cellIs" priority="38" operator="greaterThanOrEqual" dxfId="0">
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="36" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="39" operator="equal" dxfId="1">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="37" operator="lessThanOrEqual" dxfId="2">
+    <cfRule type="cellIs" priority="40" operator="lessThanOrEqual" dxfId="2">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="24">
-    <dataValidation sqref="K2:K6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+  <dataValidations count="29">
+    <dataValidation sqref="T2:T6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$A$2:$A$6</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+    <dataValidation sqref="U2:U6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$B$2:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$C$2:$C$5</formula1>
+    <dataValidation sqref="J2:J6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$C$2:$C$4</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$D$2:$D$4</formula1>
+    <dataValidation sqref="K2:K6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$D$2:$D$5</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+    <dataValidation sqref="L2:L6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$E$2:$E$4</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$F$2:$F$4</formula1>
-    </dataValidation>
-    <dataValidation sqref="Q2:Q6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$G$2:$G$4</formula1>
+    <dataValidation sqref="M2:M6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$F$2:$F$5</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$H$2:$H$4</formula1>
+      <formula1>='下拉选项'!$G$2:$G$2</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+    <dataValidation sqref="V2:V6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$H$2:$H$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$I$2:$I$4</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$J$2:$J$5</formula1>
+    <dataValidation sqref="X2:X6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$J$2:$J$4</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+    <dataValidation sqref="Y2:Y6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$K$2:$K$4</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$L$2:$L$6</formula1>
+    <dataValidation sqref="Z2:Z6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$L$2:$L$4</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$M$2:$M$6</formula1>
+    <dataValidation sqref="AA2:AA6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$M$2:$M$4</formula1>
     </dataValidation>
-    <dataValidation sqref="X2:X6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+    <dataValidation sqref="AB2:AB6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$N$2:$N$4</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$O$2:$O$4</formula1>
+    <dataValidation sqref="AC2:AC6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$O$2:$O$5</formula1>
     </dataValidation>
-    <dataValidation sqref="Z2:Z6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+    <dataValidation sqref="AD2:AD6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$P$2:$P$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$Q$2:$Q$3</formula1>
+    <dataValidation sqref="AE2:AE6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$Q$2:$Q$6</formula1>
     </dataValidation>
-    <dataValidation sqref="AB2:AB6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$R$2:$R$10</formula1>
+    <dataValidation sqref="AF2:AF6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$R$2:$R$6</formula1>
     </dataValidation>
     <dataValidation sqref="AG2:AG6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
       <formula1>='下拉选项'!$S$2:$S$4</formula1>
@@ -1589,16 +1933,31 @@
       <formula1>='下拉选项'!$T$2:$T$4</formula1>
     </dataValidation>
     <dataValidation sqref="AI2:AI6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$U$2:$U$6</formula1>
+      <formula1>='下拉选项'!$U$2:$U$4</formula1>
     </dataValidation>
     <dataValidation sqref="AJ2:AJ6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$V$2:$V$5</formula1>
+      <formula1>='下拉选项'!$V$2:$V$3</formula1>
     </dataValidation>
     <dataValidation sqref="AK2:AK6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$W$2:$W$3</formula1>
+      <formula1>='下拉选项'!$W$2:$W$10</formula1>
     </dataValidation>
-    <dataValidation sqref="AL2:AL6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
-      <formula1>='下拉选项'!$X$2:$X$5</formula1>
+    <dataValidation sqref="AP2:AP6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$X$2:$X$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AQ2:AQ6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$Y$2:$Y$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AR2:AR6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$Z$2:$Z$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="AS2:AS6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$AA$2:$AA$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="AT2:AT6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$AB$2:$AB$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="AU2:AU6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="请从下拉列表中选择中文选项，或留空。" promptTitle="结构化复核" prompt="请用下拉选择，保证能被脚本统计。" type="list">
+      <formula1>='下拉选项'!$AC$2:$AC$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1612,7 +1971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1621,7 +1980,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
@@ -1639,6 +1998,11 @@
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1654,110 +2018,135 @@
       </c>
       <c r="C1" s="10" t="inlineStr">
         <is>
+          <t>是否有完整题目上下文</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>题目摘要是否足够评分</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>是否需要查看完整题面才能评分</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>题目摘要来源</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>当前AIChat回复字段说明</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
           <t>上下文是否足够</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>识别当前缺失桥是否准确（0/1/2）</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
         <is>
           <t>回复是否基于当前材料（0/1/2）</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>脚手架是否合适（0/1/2）</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>是否控制关键桥泄露（0/1/2）</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>下一步是否清楚（0/1/2）</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>是否单焦点连贯（0/1/2）</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="O1" s="10" t="inlineStr">
         <is>
           <t>微例是否围绕桥梁（0/1/2/不适用）</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="P1" s="10" t="inlineStr">
         <is>
           <t>微例适用性</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="Q1" s="10" t="inlineStr">
         <is>
           <t>泄露标签</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="R1" s="10" t="inlineStr">
         <is>
           <t>总体质量（1-5）</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="S1" s="10" t="inlineStr">
         <is>
           <t>是否愿意给学生看</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="T1" s="10" t="inlineStr">
         <is>
           <t>学生回答负担</t>
         </is>
       </c>
-      <c r="P1" s="10" t="inlineStr">
+      <c r="U1" s="10" t="inlineStr">
         <is>
           <t>复核信心</t>
         </is>
       </c>
-      <c r="Q1" s="10" t="inlineStr">
+      <c r="V1" s="10" t="inlineStr">
         <is>
           <t>是否需要讨论</t>
         </is>
       </c>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="W1" s="10" t="inlineStr">
         <is>
           <t>缺失桥家族（中文）</t>
         </is>
       </c>
-      <c r="S1" s="10" t="inlineStr">
+      <c r="X1" s="10" t="inlineStr">
         <is>
           <t>是否匹配现有taxonomy</t>
         </is>
       </c>
-      <c r="T1" s="10" t="inlineStr">
+      <c r="Y1" s="10" t="inlineStr">
         <is>
           <t>新桥候选（如无填“无”）</t>
         </is>
       </c>
-      <c r="U1" s="10" t="inlineStr">
+      <c r="Z1" s="10" t="inlineStr">
         <is>
           <t>观察到的下一轮进展</t>
         </is>
       </c>
-      <c r="V1" s="10" t="inlineStr">
+      <c r="AA1" s="10" t="inlineStr">
         <is>
           <t>是否同意AI预标注</t>
         </is>
       </c>
-      <c r="W1" s="10" t="inlineStr">
+      <c r="AB1" s="10" t="inlineStr">
         <is>
           <t>是否需要裁决</t>
         </is>
       </c>
-      <c r="X1" s="10" t="inlineStr">
+      <c r="AC1" s="10" t="inlineStr">
         <is>
           <t>知情/报告门</t>
         </is>
@@ -1776,110 +2165,135 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>足够</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>线上AIChat元数据</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>线上已展示回复，观察项，非实验条件</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>足够</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>适用</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>无泄露</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>二分检查语义桥</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>有进展</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>同意</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>待完成</t>
         </is>
@@ -1898,110 +2312,130 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>部分足够</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>教练人工改写</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>部分足够</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>轻微关键桥泄露</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>DP状态/转移桥</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>有：见教练备注</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>部分进展</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>部分同意</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>可报告</t>
         </is>
@@ -2020,100 +2454,120 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>不足</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>题目上下文摘要</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>不足</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>不清楚</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>重大关键桥泄露</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>贡献/差分汇总桥</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>不确定</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>不确定：见教练备注</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>无进展</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>不同意</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>不可报告</t>
         </is>
@@ -2130,42 +2584,52 @@
           <t>因隐私风险排除</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>不确定</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>不清楚</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>答案或代码泄露</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>数据结构语义桥</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>不清楚</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>已退出</t>
         </is>
@@ -2177,50 +2641,50 @@
           <t>因上下文不足排除</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>上下文不足未判断</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>图/树遍历桥</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>不可用</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="R7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>调试定位桥</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="R8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>实现边界桥</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="R9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>上下文不足/澄清优先</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="R10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>其他/不确定</t>
         </is>

</xml_diff>